<commit_message>
feat(excel-splitter): add computed_columns config option
Support formula-based computed columns that are calculated after
splitting and merging, instead of being split proportionally.

- Add formula engine: tokenizer (longest-match for column names with
  parentheses), recursive-descent parser, AST evaluator
- computed_columns config: dict mapping name -> formula, evaluated
  sequentially in definition order
- Formula references must be in splitting_columns or earlier computed
  columns (circular dependency prevention)
- Only split rows are recomputed; unsplit rows keep source values
- Per-source-row verification: sum of computed column across split
  result rows must match source row's original value
- Update config.yaml: move 福利前工资合计/税前应发工资总额(不含差补)/实发工资
  from splitting_columns to computed_columns

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cursor/excel-splitter/input/项目成本.xlsx
+++ b/cursor/excel-splitter/input/项目成本.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255" firstSheet="1"/>
+    <workbookView windowWidth="28800" windowHeight="12255" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="输入-工时表" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="72">
   <si>
     <t>姓名</t>
   </si>
@@ -120,15 +120,12 @@
     <t>募投43</t>
   </si>
   <si>
-    <t>募投53</t>
+    <t>募投5</t>
   </si>
   <si>
     <t>募投44</t>
   </si>
   <si>
-    <t>募投55</t>
-  </si>
-  <si>
     <t>重庆分6</t>
   </si>
   <si>
@@ -184,6 +181,21 @@
   </si>
   <si>
     <t>岗位工资</t>
+  </si>
+  <si>
+    <t>福利前工资合计</t>
+  </si>
+  <si>
+    <t>用餐补助</t>
+  </si>
+  <si>
+    <t>税前应发工资总额(不含差补)</t>
+  </si>
+  <si>
+    <t>差旅补助</t>
+  </si>
+  <si>
+    <t>实发工资</t>
   </si>
   <si>
     <t>工资所属单位</t>
@@ -1538,95 +1550,95 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11">
         <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12">
         <v>7</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18">
         <v>5</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1662,17 +1674,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="7"/>
   <cols>
     <col min="4" max="5" width="9" style="1"/>
-    <col min="6" max="6" width="10.2166666666667" customWidth="1"/>
-    <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="14.5583333333333" customWidth="1"/>
-    <col min="9" max="9" width="12.4416666666667" customWidth="1"/>
+    <col min="6" max="7" width="15.25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.75" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9" style="1"/>
+    <col min="11" max="11" width="10.2166666666667" customWidth="1"/>
+    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="13" max="13" width="14.5583333333333" customWidth="1"/>
+    <col min="14" max="14" width="12.4416666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:16">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1680,34 +1696,49 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
+        <v>55</v>
+      </c>
+      <c r="P1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1715,7 +1746,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D2" s="1">
         <v>1000</v>
@@ -1723,23 +1754,41 @@
       <c r="E2" s="1">
         <v>300</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1">
+        <f t="shared" ref="F2:F8" si="0">D2+E2</f>
+        <v>1300</v>
+      </c>
+      <c r="G2" s="1">
+        <v>200</v>
+      </c>
+      <c r="H2" s="1">
+        <f t="shared" ref="H2:H8" si="1">F2+G2</f>
+        <v>1500</v>
+      </c>
+      <c r="I2" s="1">
+        <v>100</v>
+      </c>
+      <c r="J2" s="1">
+        <f t="shared" ref="J2:J8" si="2">H2+I2</f>
+        <v>1600</v>
+      </c>
+      <c r="K2" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
-        <v>53</v>
-      </c>
-      <c r="I2">
+      <c r="M2" t="s">
+        <v>57</v>
+      </c>
+      <c r="N2">
         <v>21</v>
       </c>
-      <c r="J2" t="s">
+      <c r="O2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1747,7 +1796,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D3" s="3">
         <v>2000</v>
@@ -1755,23 +1804,41 @@
       <c r="E3" s="1">
         <v>100</v>
       </c>
-      <c r="F3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="F3" s="1">
+        <f t="shared" si="0"/>
+        <v>2100</v>
+      </c>
+      <c r="G3" s="1">
+        <v>200</v>
+      </c>
+      <c r="H3" s="1">
+        <f t="shared" si="1"/>
+        <v>2300</v>
+      </c>
+      <c r="I3" s="1">
+        <v>101</v>
+      </c>
+      <c r="J3" s="1">
+        <f t="shared" si="2"/>
+        <v>2401</v>
+      </c>
+      <c r="K3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H3" t="s">
-        <v>56</v>
-      </c>
-      <c r="I3">
+      <c r="M3" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3">
         <v>20</v>
       </c>
-      <c r="J3" t="s">
+      <c r="O3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1779,36 +1846,57 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D4" s="1">
         <v>3000</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E4" s="1">
+        <v>200</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>3200</v>
+      </c>
+      <c r="G4" s="1">
+        <v>200</v>
+      </c>
+      <c r="H4" s="1">
+        <f t="shared" si="1"/>
+        <v>3400</v>
+      </c>
+      <c r="I4" s="1">
+        <v>102</v>
+      </c>
+      <c r="J4" s="1">
+        <f t="shared" si="2"/>
+        <v>3502</v>
+      </c>
+      <c r="K4" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4">
+      <c r="M4" t="s">
+        <v>62</v>
+      </c>
+      <c r="N4">
         <v>22</v>
       </c>
-      <c r="J4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="O4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D5" s="1">
         <v>4000</v>
@@ -1816,31 +1904,49 @@
       <c r="E5" s="1">
         <v>1000</v>
       </c>
-      <c r="F5" t="s">
-        <v>62</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5">
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
+      <c r="G5" s="1">
+        <v>200</v>
+      </c>
+      <c r="H5" s="1">
+        <f t="shared" si="1"/>
+        <v>5200</v>
+      </c>
+      <c r="I5" s="1">
+        <v>103</v>
+      </c>
+      <c r="J5" s="1">
+        <f t="shared" si="2"/>
+        <v>5303</v>
+      </c>
+      <c r="K5" t="s">
+        <v>66</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5">
         <v>10</v>
       </c>
-      <c r="J5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="O5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D6" s="1">
         <v>5000</v>
@@ -1848,23 +1954,41 @@
       <c r="E6" s="1">
         <v>2000</v>
       </c>
-      <c r="F6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6">
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+        <v>7000</v>
+      </c>
+      <c r="G6" s="1">
+        <v>200</v>
+      </c>
+      <c r="H6" s="1">
+        <f t="shared" si="1"/>
+        <v>7200</v>
+      </c>
+      <c r="I6" s="1">
+        <v>104</v>
+      </c>
+      <c r="J6" s="1">
+        <f t="shared" si="2"/>
+        <v>7304</v>
+      </c>
+      <c r="K6" t="s">
+        <v>71</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6">
         <v>15</v>
       </c>
-      <c r="J6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="O6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1872,7 +1996,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D7" s="3">
         <v>2000</v>
@@ -1880,23 +2004,41 @@
       <c r="E7" s="1">
         <v>100</v>
       </c>
-      <c r="F7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="2" t="s">
+      <c r="F7" s="1">
+        <f t="shared" si="0"/>
+        <v>2100</v>
+      </c>
+      <c r="G7" s="1">
+        <v>200</v>
+      </c>
+      <c r="H7" s="1">
+        <f t="shared" si="1"/>
+        <v>2300</v>
+      </c>
+      <c r="I7" s="1">
+        <v>105</v>
+      </c>
+      <c r="J7" s="1">
+        <f t="shared" si="2"/>
+        <v>2405</v>
+      </c>
+      <c r="K7" t="s">
+        <v>59</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H7" t="s">
-        <v>56</v>
-      </c>
-      <c r="I7">
+      <c r="M7" t="s">
+        <v>60</v>
+      </c>
+      <c r="N7">
         <v>20</v>
       </c>
-      <c r="J7" t="s">
+      <c r="O7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1904,7 +2046,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D8" s="3">
         <v>2000</v>
@@ -1912,19 +2054,37 @@
       <c r="E8" s="1">
         <v>100</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+        <v>2100</v>
+      </c>
+      <c r="G8" s="1">
+        <v>200</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" si="1"/>
+        <v>2300</v>
+      </c>
+      <c r="I8" s="1">
+        <v>106</v>
+      </c>
+      <c r="J8" s="1">
+        <f t="shared" si="2"/>
+        <v>2406</v>
+      </c>
+      <c r="K8" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" t="s">
-        <v>53</v>
-      </c>
-      <c r="I8">
+      <c r="L8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M8" t="s">
+        <v>57</v>
+      </c>
+      <c r="N8">
         <v>20</v>
       </c>
-      <c r="J8" t="s">
+      <c r="O8" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(excel-splitter): update input data
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cursor/excel-splitter/input/项目成本.xlsx
+++ b/cursor/excel-splitter/input/项目成本.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="74">
   <si>
     <t>姓名</t>
   </si>
@@ -75,153 +75,165 @@
     <t>CC</t>
   </si>
   <si>
+    <t>吴八</t>
+  </si>
+  <si>
+    <t>GG</t>
+  </si>
+  <si>
+    <t>公司</t>
+  </si>
+  <si>
+    <t>项目名称</t>
+  </si>
+  <si>
+    <t>支付账户</t>
+  </si>
+  <si>
+    <t>开户行</t>
+  </si>
+  <si>
+    <t>重庆分3</t>
+  </si>
+  <si>
+    <t>募投31</t>
+  </si>
+  <si>
+    <t>重庆分4</t>
+  </si>
+  <si>
+    <t>募投41</t>
+  </si>
+  <si>
+    <t>募投32</t>
+  </si>
+  <si>
+    <t>重庆分5</t>
+  </si>
+  <si>
+    <t>募投52</t>
+  </si>
+  <si>
+    <t>募投33</t>
+  </si>
+  <si>
+    <t>募投43</t>
+  </si>
+  <si>
+    <t>募投5</t>
+  </si>
+  <si>
+    <t>募投44</t>
+  </si>
+  <si>
+    <t>重庆分6</t>
+  </si>
+  <si>
+    <t>募投66</t>
+  </si>
+  <si>
+    <t>重庆分7</t>
+  </si>
+  <si>
+    <t>募投77</t>
+  </si>
+  <si>
+    <t>重庆分</t>
+  </si>
+  <si>
+    <t>营销中心1</t>
+  </si>
+  <si>
+    <t>营销</t>
+  </si>
+  <si>
+    <t>YX1</t>
+  </si>
+  <si>
+    <t>营销中心2</t>
+  </si>
+  <si>
+    <t>YX2</t>
+  </si>
+  <si>
+    <t>行政部</t>
+  </si>
+  <si>
+    <t>行政</t>
+  </si>
+  <si>
+    <t>XZB6</t>
+  </si>
+  <si>
+    <t>XZB7</t>
+  </si>
+  <si>
+    <t>财务部</t>
+  </si>
+  <si>
+    <t>财务</t>
+  </si>
+  <si>
+    <t>CWB</t>
+  </si>
+  <si>
+    <t>重庆分8</t>
+  </si>
+  <si>
+    <t>募投85</t>
+  </si>
+  <si>
+    <t>部门</t>
+  </si>
+  <si>
+    <t>基本工资</t>
+  </si>
+  <si>
+    <t>岗位工资</t>
+  </si>
+  <si>
+    <t>福利前工资合计</t>
+  </si>
+  <si>
+    <t>用餐补助</t>
+  </si>
+  <si>
+    <t>税前应发工资总额(不含差补)</t>
+  </si>
+  <si>
+    <t>差旅补助</t>
+  </si>
+  <si>
+    <t>实发工资</t>
+  </si>
+  <si>
+    <t>工资所属单位</t>
+  </si>
+  <si>
+    <t>分管领导</t>
+  </si>
+  <si>
+    <t>中国</t>
+  </si>
+  <si>
+    <t>研发部</t>
+  </si>
+  <si>
+    <t>美国</t>
+  </si>
+  <si>
+    <t>人事</t>
+  </si>
+  <si>
+    <t>人事部</t>
+  </si>
+  <si>
+    <t>日本</t>
+  </si>
+  <si>
     <t>销售</t>
   </si>
   <si>
-    <t>吴八</t>
-  </si>
-  <si>
-    <t>GG</t>
-  </si>
-  <si>
-    <t>公司</t>
-  </si>
-  <si>
-    <t>项目名称</t>
-  </si>
-  <si>
-    <t>支付账户</t>
-  </si>
-  <si>
-    <t>重庆分3</t>
-  </si>
-  <si>
-    <t>募投31</t>
-  </si>
-  <si>
-    <t>重庆分4</t>
-  </si>
-  <si>
-    <t>募投41</t>
-  </si>
-  <si>
-    <t>募投32</t>
-  </si>
-  <si>
-    <t>重庆分5</t>
-  </si>
-  <si>
-    <t>募投52</t>
-  </si>
-  <si>
-    <t>募投33</t>
-  </si>
-  <si>
-    <t>募投43</t>
-  </si>
-  <si>
-    <t>募投5</t>
-  </si>
-  <si>
-    <t>募投44</t>
-  </si>
-  <si>
-    <t>重庆分6</t>
-  </si>
-  <si>
-    <t>募投66</t>
-  </si>
-  <si>
-    <t>重庆分7</t>
-  </si>
-  <si>
-    <t>募投77</t>
-  </si>
-  <si>
-    <t>重庆分</t>
-  </si>
-  <si>
-    <t>营销中心1</t>
-  </si>
-  <si>
-    <t>YX1</t>
-  </si>
-  <si>
-    <t>营销中心2</t>
-  </si>
-  <si>
-    <t>YX2</t>
-  </si>
-  <si>
-    <t>行政部</t>
-  </si>
-  <si>
-    <t>XZB6</t>
-  </si>
-  <si>
-    <t>XZB7</t>
-  </si>
-  <si>
-    <t>财务部</t>
-  </si>
-  <si>
-    <t>CWB</t>
-  </si>
-  <si>
-    <t>重庆分8</t>
-  </si>
-  <si>
-    <t>募投85</t>
-  </si>
-  <si>
-    <t>部门</t>
-  </si>
-  <si>
-    <t>基本工资</t>
-  </si>
-  <si>
-    <t>岗位工资</t>
-  </si>
-  <si>
-    <t>福利前工资合计</t>
-  </si>
-  <si>
-    <t>用餐补助</t>
-  </si>
-  <si>
-    <t>税前应发工资总额(不含差补)</t>
-  </si>
-  <si>
-    <t>差旅补助</t>
-  </si>
-  <si>
-    <t>实发工资</t>
-  </si>
-  <si>
-    <t>工资所属单位</t>
-  </si>
-  <si>
-    <t>分管领导</t>
-  </si>
-  <si>
-    <t>中国</t>
-  </si>
-  <si>
-    <t>研发部</t>
-  </si>
-  <si>
-    <t>美国</t>
-  </si>
-  <si>
-    <t>人事</t>
-  </si>
-  <si>
-    <t>人事部</t>
-  </si>
-  <si>
-    <t>日本</t>
-  </si>
-  <si>
     <t>销售部</t>
   </si>
   <si>
@@ -234,9 +246,6 @@
     <t>法国</t>
   </si>
   <si>
-    <t>行政</t>
-  </si>
-  <si>
     <t>EE</t>
   </si>
   <si>
@@ -247,9 +256,6 @@
   </si>
   <si>
     <t>英国</t>
-  </si>
-  <si>
-    <t>财务</t>
   </si>
 </sst>
 </file>
@@ -1325,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D6">
         <v>3</v>
@@ -1342,7 +1348,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D7">
         <v>3</v>
@@ -1359,7 +1365,7 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D8">
         <v>3</v>
@@ -1376,7 +1382,7 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -1393,7 +1399,7 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D10">
         <v>5</v>
@@ -1404,10 +1410,10 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
         <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
@@ -1430,240 +1436,366 @@
   <sheetPr>
     <tabColor theme="8" tint="0.799981688894314"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="3"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="16.1083333333333" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22.3333333333333" style="2" customWidth="1"/>
-    <col min="3" max="3" width="42" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.55833333333333" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="2"/>
+    <col min="2" max="3" width="22.3333333333333" style="2" customWidth="1"/>
+    <col min="4" max="4" width="42" style="2" customWidth="1"/>
+    <col min="5" max="5" width="9.55833333333333" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.25" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="F2" s="2" t="str">
+        <f t="shared" ref="F2:F18" si="0">E2&amp;"开户行"</f>
+        <v>募投31开户行</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="F3" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投41开户行</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="F4" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投32开户行</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="F5" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投52开户行</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="F6" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投33开户行</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B7">
         <v>3</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="F7" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投43开户行</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B8">
         <v>3</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="F8" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投5开户行</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="F9" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投44开户行</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B10">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="F10" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投5开户行</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B11">
         <v>6</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="F11" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投66开户行</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B12">
         <v>7</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="F12" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投77开户行</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>YX1开户行</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="C14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>YX2开户行</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>XZB6开户行</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>XZB7开户行</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>CWB开户行</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>5</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>45</v>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>募投85开户行</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C3">
+  <conditionalFormatting sqref="D3">
     <cfRule type="duplicateValues" dxfId="0" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4">
+  <conditionalFormatting sqref="D4">
     <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C7">
+  <conditionalFormatting sqref="D7">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C8">
+  <conditionalFormatting sqref="D8">
     <cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C16">
+  <conditionalFormatting sqref="D16">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
+  <conditionalFormatting sqref="D18">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C2 C5:C6 C9:C14 C19:C1048576">
+  <conditionalFormatting sqref="D1:D2 D5:D6 D9:D14 D19:D1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C15 C17">
+  <conditionalFormatting sqref="D15 D17">
     <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1696,34 +1828,34 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K1" t="s">
         <v>2</v>
       </c>
       <c r="L1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="M1" t="s">
         <v>3</v>
@@ -1732,10 +1864,10 @@
         <v>4</v>
       </c>
       <c r="O1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="P1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -1746,7 +1878,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D2" s="1">
         <v>1000</v>
@@ -1779,7 +1911,7 @@
         <v>19</v>
       </c>
       <c r="M2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="N2">
         <v>21</v>
@@ -1796,7 +1928,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D3" s="3">
         <v>2000</v>
@@ -1823,13 +1955,13 @@
         <v>2401</v>
       </c>
       <c r="K3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="M3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="N3">
         <v>20</v>
@@ -1846,7 +1978,7 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D4" s="1">
         <v>3000</v>
@@ -1873,30 +2005,30 @@
         <v>3502</v>
       </c>
       <c r="K4" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N4">
         <v>22</v>
       </c>
       <c r="O4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D5" s="1">
         <v>4000</v>
@@ -1923,30 +2055,30 @@
         <v>5303</v>
       </c>
       <c r="K5" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N5">
         <v>10</v>
       </c>
       <c r="O5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D6" s="1">
         <v>5000</v>
@@ -1973,19 +2105,19 @@
         <v>7304</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N6">
         <v>15</v>
       </c>
       <c r="O6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1996,7 +2128,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D7" s="3">
         <v>2000</v>
@@ -2023,13 +2155,13 @@
         <v>2405</v>
       </c>
       <c r="K7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="M7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="N7">
         <v>20</v>
@@ -2040,13 +2172,13 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D8" s="3">
         <v>2000</v>
@@ -2076,10 +2208,10 @@
         <v>8</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="M8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="N8">
         <v>20</v>

</xml_diff>